<commit_message>
progress: 68 village workbooks (sivaramans-llin 2026-10-10T19:00:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Pondavakkam_13.469251_79.994996.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Pondavakkam_13.469251_79.994996.xlsx
@@ -4778,6 +4778,11 @@
           <t>43</t>
         </is>
       </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
@@ -4785,6 +4790,11 @@
           <t>430</t>
         </is>
       </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>1, 10, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
@@ -4792,6 +4802,11 @@
           <t>431</t>
         </is>
       </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
@@ -4799,6 +4814,11 @@
           <t>432</t>
         </is>
       </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21, 22, 23, 24, 25, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
@@ -4806,11 +4826,21 @@
           <t>433</t>
         </is>
       </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
         <is>
           <t>434</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>

</xml_diff>